<commit_message>
Login: gast-toegang zonder login
</commit_message>
<xml_diff>
--- a/MANUAL.xlsx
+++ b/MANUAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://winsolgroup-my.sharepoint.com/personal/gwenn_vanthournout_winsol_eu/Documents/_Gwenn/DOCS/AI/SOCRATES_WEB_DEV/frontend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="167" documentId="8_{AEEDC2F3-0F41-481B-990B-CA8573AB31BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A0E43C1-A2FA-44FA-B144-68423DF468E9}"/>
+  <xr:revisionPtr revIDLastSave="173" documentId="8_{AEEDC2F3-0F41-481B-990B-CA8573AB31BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3F3E94F-A848-4516-92B5-627E75EB805E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E13C84A-EF44-4272-976B-DB216750A179}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E13C84A-EF44-4272-976B-DB216750A179}"/>
   </bookViews>
   <sheets>
     <sheet name="SCREEN-PRODUCTSTORING" sheetId="1" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="94">
   <si>
     <t>START: Minimale nodig info</t>
   </si>
@@ -290,9 +290,6 @@
     <t>SO! Screen - Maestria WT</t>
   </si>
   <si>
-    <t>SO! Screen - Kalibratie</t>
-  </si>
-  <si>
     <t>MANUAL</t>
   </si>
   <si>
@@ -354,6 +351,12 @@
   </si>
   <si>
     <t>MC01, MC02, MC03, MC04, MC05, MC06, MC07, MC08</t>
+  </si>
+  <si>
+    <t>SolarFix - Winsol Silent Motor</t>
+  </si>
+  <si>
+    <t>SolarFix - Somfy Motor</t>
   </si>
 </sst>
 </file>
@@ -808,7 +811,7 @@
       </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>2</v>
@@ -828,10 +831,10 @@
       <c r="M1" s="12"/>
       <c r="N1" s="12"/>
       <c r="O1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P1" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>74</v>
       </c>
       <c r="Q1" s="12" t="s">
         <v>6</v>
@@ -854,29 +857,29 @@
         <v>70</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>38</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="M2" s="9"/>
       <c r="N2" s="9"/>
       <c r="O2" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="P2" s="7" t="s">
         <v>77</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -885,30 +888,30 @@
         <v>9</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="7" t="s">
         <v>39</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
       <c r="N3" s="9"/>
       <c r="O3" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="P3" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -916,28 +919,31 @@
       <c r="D4" s="7" t="s">
         <v>10</v>
       </c>
+      <c r="E4" s="7" t="s">
+        <v>93</v>
+      </c>
       <c r="F4" s="8"/>
       <c r="G4" s="7" t="s">
         <v>40</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K4" s="9"/>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
       <c r="N4" s="9"/>
       <c r="O4" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P4" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -951,23 +957,23 @@
         <v>41</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
       <c r="O5" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="P5" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -981,23 +987,23 @@
         <v>42</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K6" s="9"/>
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
       <c r="O6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="P6" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1011,23 +1017,23 @@
         <v>43</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
       <c r="O7" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1041,23 +1047,23 @@
         <v>44</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
       <c r="N8" s="9"/>
       <c r="O8" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1071,23 +1077,23 @@
         <v>45</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="9"/>
       <c r="O9" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>